<commit_message>
Bugfix - missing highlighting in negative xlsx files
</commit_message>
<xml_diff>
--- a/rules/CORE-000262/negative/01/data/unit-test-coreid-CG0226-negative 1.xlsx
+++ b/rules/CORE-000262/negative/01/data/unit-test-coreid-CG0226-negative 1.xlsx
@@ -37,7 +37,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" mc:Ignorable="x14ac">
   <numFmts count="0"/>
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <name val="Calibri"/>
@@ -60,8 +60,12 @@
       <name val="Calibri"/>
       <i/>
     </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none">
         <bgColor/>
@@ -75,6 +79,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFFFCC"/>
+        <bgColor/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
         <bgColor/>
       </patternFill>
     </fill>
@@ -98,13 +108,14 @@
   <cellStyleXfs>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="1" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -447,10 +458,10 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="str">
+      <c r="A2" s="4" t="str">
         <v>sdtmig</v>
       </c>
-      <c r="B2" s="2" t="str">
+      <c r="B2" s="4" t="str">
         <v>3-4</v>
       </c>
     </row>
@@ -474,18 +485,18 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="str">
+      <c r="A2" s="4" t="str">
         <v>dm.xpt</v>
       </c>
-      <c r="B2" s="2" t="str">
+      <c r="B2" s="4" t="str">
         <v>Demographics</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="str">
+      <c r="A3" s="4" t="str">
         <v>cm.xpt</v>
       </c>
-      <c r="B3" s="2" t="str">
+      <c r="B3" s="4" t="str">
         <v>Concomitant/Prior Medications</v>
       </c>
     </row>
@@ -521,16 +532,16 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2">
+      <c r="A2" s="4">
         <v>1</v>
       </c>
-      <c r="B2" s="2" t="str">
+      <c r="B2" s="4" t="str">
         <v>dm.xpt</v>
       </c>
-      <c r="C2" s="2" t="str">
+      <c r="C2" s="4" t="str">
         <v>Record</v>
       </c>
-      <c r="D2" s="2">
+      <c r="D2" s="4">
         <v>5</v>
       </c>
       <c r="E2" s="4" t="str">
@@ -538,16 +549,16 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2">
+      <c r="A3" s="4">
         <v>1</v>
       </c>
-      <c r="B3" s="2" t="str">
+      <c r="B3" s="4" t="str">
         <v>cm.xpt</v>
       </c>
-      <c r="C3" s="2" t="str">
+      <c r="C3" s="4" t="str">
         <v>Record</v>
       </c>
-      <c r="D3" s="2">
+      <c r="D3" s="4">
         <v>5</v>
       </c>
       <c r="E3" s="4" t="str">
@@ -558,16 +569,16 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="2">
+      <c r="A4" s="4">
         <v>2</v>
       </c>
-      <c r="B4" s="2" t="str">
+      <c r="B4" s="4" t="str">
         <v>dm.xpt</v>
       </c>
-      <c r="C4" s="2" t="str">
+      <c r="C4" s="4" t="str">
         <v>Record</v>
       </c>
-      <c r="D4" s="2">
+      <c r="D4" s="4">
         <v>7</v>
       </c>
       <c r="E4" s="4" t="str">
@@ -575,16 +586,16 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="2">
+      <c r="A5" s="4">
         <v>2</v>
       </c>
-      <c r="B5" s="2" t="str">
+      <c r="B5" s="4" t="str">
         <v>cm.xpt</v>
       </c>
-      <c r="C5" s="2" t="str">
+      <c r="C5" s="4" t="str">
         <v>Record</v>
       </c>
-      <c r="D5" s="2">
+      <c r="D5" s="4">
         <v>7</v>
       </c>
       <c r="E5" s="4" t="str">
@@ -595,16 +606,16 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="2">
+      <c r="A6" s="4">
         <v>3</v>
       </c>
-      <c r="B6" s="2" t="str">
+      <c r="B6" s="4" t="str">
         <v>dm.xpt</v>
       </c>
-      <c r="C6" s="2" t="str">
+      <c r="C6" s="4" t="str">
         <v>Record</v>
       </c>
-      <c r="D6" s="2">
+      <c r="D6" s="4">
         <v>9</v>
       </c>
       <c r="E6" s="4" t="str">
@@ -612,16 +623,16 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="2">
+      <c r="A7" s="4">
         <v>3</v>
       </c>
-      <c r="B7" s="2" t="str">
+      <c r="B7" s="4" t="str">
         <v>cm.xpt</v>
       </c>
-      <c r="C7" s="2" t="str">
+      <c r="C7" s="4" t="str">
         <v>Record</v>
       </c>
-      <c r="D7" s="2">
+      <c r="D7" s="4">
         <v>9</v>
       </c>
       <c r="E7" s="4" t="str">
@@ -632,16 +643,16 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="2">
+      <c r="A8" s="4">
         <v>4</v>
       </c>
-      <c r="B8" s="2" t="str">
+      <c r="B8" s="4" t="str">
         <v>dm.xpt</v>
       </c>
-      <c r="C8" s="2" t="str">
+      <c r="C8" s="4" t="str">
         <v>Record</v>
       </c>
-      <c r="D8" s="2">
+      <c r="D8" s="4">
         <v>13</v>
       </c>
       <c r="E8" s="4" t="str">
@@ -649,16 +660,16 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="2">
+      <c r="A9" s="4">
         <v>4</v>
       </c>
-      <c r="B9" s="2" t="str">
+      <c r="B9" s="4" t="str">
         <v>cm.xpt</v>
       </c>
-      <c r="C9" s="2" t="str">
+      <c r="C9" s="4" t="str">
         <v>Record</v>
       </c>
-      <c r="D9" s="2">
+      <c r="D9" s="4">
         <v>13</v>
       </c>
       <c r="E9" s="4" t="str">
@@ -1012,7 +1023,7 @@
       <c r="D5" s="4">
         <v>1115</v>
       </c>
-      <c r="E5" s="4" t="str">
+      <c r="E5" s="6" t="str">
         <v/>
       </c>
       <c r="F5" s="4" t="str">
@@ -1172,7 +1183,7 @@
       <c r="D7" s="4">
         <v>1302</v>
       </c>
-      <c r="E7" s="4" t="str">
+      <c r="E7" s="6" t="str">
         <v/>
       </c>
       <c r="F7" s="4" t="str">
@@ -1332,7 +1343,7 @@
       <c r="D9" s="4">
         <v>1383</v>
       </c>
-      <c r="E9" s="4" t="str">
+      <c r="E9" s="6" t="str">
         <v/>
       </c>
       <c r="F9" s="4" t="str">
@@ -1652,7 +1663,7 @@
       <c r="D13" s="4">
         <v>1087</v>
       </c>
-      <c r="E13" s="4" t="str">
+      <c r="E13" s="6" t="str">
         <v/>
       </c>
       <c r="F13" s="4" t="str">
@@ -2068,7 +2079,7 @@
       <c r="O5" s="4" t="str">
         <v/>
       </c>
-      <c r="P5" s="4" t="str">
+      <c r="P5" s="6" t="str">
         <v>ONGOING</v>
       </c>
       <c r="Q5" s="4" t="str">
@@ -2174,7 +2185,7 @@
       <c r="O7" s="4" t="str">
         <v/>
       </c>
-      <c r="P7" s="4" t="str">
+      <c r="P7" s="6" t="str">
         <v>ONGOING</v>
       </c>
       <c r="Q7" s="4" t="str">
@@ -2280,7 +2291,7 @@
       <c r="O9" s="4">
         <v>1</v>
       </c>
-      <c r="P9" s="4" t="str">
+      <c r="P9" s="6" t="str">
         <v>BEFORE</v>
       </c>
       <c r="Q9" s="4" t="str">
@@ -2492,7 +2503,7 @@
       <c r="O13" s="4">
         <v>181</v>
       </c>
-      <c r="P13" s="4" t="str">
+      <c r="P13" s="6" t="str">
         <v>AFTER</v>
       </c>
       <c r="Q13" s="4" t="str">

</xml_diff>

<commit_message>
Bugfix - added the correct validating variable to the YAML file and applied the right variable order in the XLSX files
</commit_message>
<xml_diff>
--- a/rules/CORE-000262/negative/01/data/unit-test-coreid-CG0226-negative 1.xlsx
+++ b/rules/CORE-000262/negative/01/data/unit-test-coreid-CG0226-negative 1.xlsx
@@ -37,7 +37,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" mc:Ignorable="x14ac">
   <numFmts count="0"/>
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <name val="Calibri"/>
@@ -63,9 +63,18 @@
     <font>
       <sz val="11"/>
       <name val="Calibri"/>
+      <i/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="6">
     <fill>
       <patternFill patternType="none">
         <bgColor/>
@@ -79,6 +88,18 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFFFCC"/>
+        <bgColor/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFCC"/>
+        <bgColor/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
         <bgColor/>
       </patternFill>
     </fill>
@@ -108,7 +129,7 @@
   <cellStyleXfs>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="1" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
@@ -116,6 +137,8 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -536,7 +559,7 @@
         <v>1</v>
       </c>
       <c r="B2" s="4" t="str">
-        <v>dm.xpt</v>
+        <v>cm.xpt</v>
       </c>
       <c r="C2" s="4" t="str">
         <v>Record</v>
@@ -545,7 +568,10 @@
         <v>5</v>
       </c>
       <c r="E2" s="4" t="str">
-        <v>RFSTDTC</v>
+        <v>CMSTRF</v>
+      </c>
+      <c r="F2" s="4" t="str">
+        <v>ONGOING</v>
       </c>
     </row>
     <row r="3">
@@ -553,7 +579,7 @@
         <v>1</v>
       </c>
       <c r="B3" s="4" t="str">
-        <v>cm.xpt</v>
+        <v>dm.xpt</v>
       </c>
       <c r="C3" s="4" t="str">
         <v>Record</v>
@@ -562,10 +588,7 @@
         <v>5</v>
       </c>
       <c r="E3" s="4" t="str">
-        <v>CMSTRF</v>
-      </c>
-      <c r="F3" s="4" t="str">
-        <v>ONGOING</v>
+        <v>RFSTDTC</v>
       </c>
     </row>
     <row r="4">
@@ -573,7 +596,7 @@
         <v>2</v>
       </c>
       <c r="B4" s="4" t="str">
-        <v>dm.xpt</v>
+        <v>cm.xpt</v>
       </c>
       <c r="C4" s="4" t="str">
         <v>Record</v>
@@ -582,7 +605,10 @@
         <v>7</v>
       </c>
       <c r="E4" s="4" t="str">
-        <v>RFSTDTC</v>
+        <v>CMSTRF</v>
+      </c>
+      <c r="F4" s="4" t="str">
+        <v>ONGOING</v>
       </c>
     </row>
     <row r="5">
@@ -590,7 +616,7 @@
         <v>2</v>
       </c>
       <c r="B5" s="4" t="str">
-        <v>cm.xpt</v>
+        <v>dm.xpt</v>
       </c>
       <c r="C5" s="4" t="str">
         <v>Record</v>
@@ -599,10 +625,7 @@
         <v>7</v>
       </c>
       <c r="E5" s="4" t="str">
-        <v>CMSTRF</v>
-      </c>
-      <c r="F5" s="4" t="str">
-        <v>ONGOING</v>
+        <v>RFSTDTC</v>
       </c>
     </row>
     <row r="6">
@@ -610,7 +633,7 @@
         <v>3</v>
       </c>
       <c r="B6" s="4" t="str">
-        <v>dm.xpt</v>
+        <v>cm.xpt</v>
       </c>
       <c r="C6" s="4" t="str">
         <v>Record</v>
@@ -619,7 +642,10 @@
         <v>9</v>
       </c>
       <c r="E6" s="4" t="str">
-        <v>RFSTDTC</v>
+        <v>CMSTRF</v>
+      </c>
+      <c r="F6" s="4" t="str">
+        <v>BEFORE</v>
       </c>
     </row>
     <row r="7">
@@ -627,7 +653,7 @@
         <v>3</v>
       </c>
       <c r="B7" s="4" t="str">
-        <v>cm.xpt</v>
+        <v>dm.xpt</v>
       </c>
       <c r="C7" s="4" t="str">
         <v>Record</v>
@@ -636,10 +662,7 @@
         <v>9</v>
       </c>
       <c r="E7" s="4" t="str">
-        <v>CMSTRF</v>
-      </c>
-      <c r="F7" s="4" t="str">
-        <v>BEFORE</v>
+        <v>RFSTDTC</v>
       </c>
     </row>
     <row r="8">
@@ -647,7 +670,7 @@
         <v>4</v>
       </c>
       <c r="B8" s="4" t="str">
-        <v>dm.xpt</v>
+        <v>cm.xpt</v>
       </c>
       <c r="C8" s="4" t="str">
         <v>Record</v>
@@ -656,7 +679,10 @@
         <v>13</v>
       </c>
       <c r="E8" s="4" t="str">
-        <v>RFSTDTC</v>
+        <v>CMSTRF</v>
+      </c>
+      <c r="F8" s="4" t="str">
+        <v>AFTER</v>
       </c>
     </row>
     <row r="9">
@@ -664,7 +690,7 @@
         <v>4</v>
       </c>
       <c r="B9" s="4" t="str">
-        <v>cm.xpt</v>
+        <v>dm.xpt</v>
       </c>
       <c r="C9" s="4" t="str">
         <v>Record</v>
@@ -673,10 +699,7 @@
         <v>13</v>
       </c>
       <c r="E9" s="4" t="str">
-        <v>CMSTRF</v>
-      </c>
-      <c r="F9" s="4" t="str">
-        <v>AFTER</v>
+        <v>RFSTDTC</v>
       </c>
     </row>
   </sheetData>
@@ -774,239 +797,239 @@
       <c r="A2" s="5" t="str">
         <v>Study Identifier</v>
       </c>
-      <c r="B2" s="5" t="str">
+      <c r="B2" s="6" t="str">
         <v>Domain Abbreviation</v>
       </c>
-      <c r="C2" s="5" t="str">
+      <c r="C2" s="6" t="str">
         <v>Unique Subject Identifier</v>
       </c>
-      <c r="D2" s="5" t="str">
+      <c r="D2" s="6" t="str">
         <v>Subject Identifier for the Study</v>
       </c>
-      <c r="E2" s="5" t="str">
+      <c r="E2" s="6" t="str">
         <v>Subject Reference Start Date/Time</v>
       </c>
-      <c r="F2" s="5" t="str">
+      <c r="F2" s="6" t="str">
         <v>Subject Reference End Date/Time</v>
       </c>
-      <c r="G2" s="5" t="str">
+      <c r="G2" s="6" t="str">
         <v>Date/Time of First Study Treatment</v>
       </c>
-      <c r="H2" s="5" t="str">
+      <c r="H2" s="6" t="str">
         <v>Date/Time of Last Study Treatment</v>
       </c>
-      <c r="I2" s="5" t="str">
+      <c r="I2" s="6" t="str">
         <v>Date/Time of Informed Consent</v>
       </c>
-      <c r="J2" s="5" t="str">
+      <c r="J2" s="6" t="str">
         <v>Date/Time of End of Participation</v>
       </c>
-      <c r="K2" s="5" t="str">
+      <c r="K2" s="6" t="str">
         <v>Date/Time of Death</v>
       </c>
-      <c r="L2" s="5" t="str">
+      <c r="L2" s="6" t="str">
         <v>Subject Death Flag</v>
       </c>
-      <c r="M2" s="5" t="str">
+      <c r="M2" s="6" t="str">
         <v>Study Site Identifier</v>
       </c>
-      <c r="N2" s="5" t="str">
+      <c r="N2" s="6" t="str">
         <v>Date/Time of Birth</v>
       </c>
-      <c r="O2" s="5" t="str">
+      <c r="O2" s="6" t="str">
         <v>Age</v>
       </c>
-      <c r="P2" s="5" t="str">
+      <c r="P2" s="6" t="str">
         <v>Age Units</v>
       </c>
-      <c r="Q2" s="5" t="str">
+      <c r="Q2" s="6" t="str">
         <v>Sex</v>
       </c>
-      <c r="R2" s="5" t="str">
+      <c r="R2" s="6" t="str">
         <v>Race</v>
       </c>
-      <c r="S2" s="5" t="str">
+      <c r="S2" s="6" t="str">
         <v>Ethnicity</v>
       </c>
-      <c r="T2" s="5" t="str">
+      <c r="T2" s="6" t="str">
         <v>Planned Arm Code</v>
       </c>
-      <c r="U2" s="5" t="str">
+      <c r="U2" s="6" t="str">
         <v>Description of Planned Arm</v>
       </c>
-      <c r="V2" s="5" t="str">
+      <c r="V2" s="6" t="str">
         <v>Actual Arm Code</v>
       </c>
-      <c r="W2" s="5" t="str">
+      <c r="W2" s="6" t="str">
         <v>Description of Actual Arm</v>
       </c>
-      <c r="X2" s="5" t="str">
+      <c r="X2" s="6" t="str">
         <v>Reason Arm and/or Actual Arm is Null</v>
       </c>
-      <c r="Y2" s="5" t="str">
+      <c r="Y2" s="6" t="str">
         <v>Description of Unplanned Actual Arm</v>
       </c>
-      <c r="Z2" s="5" t="str">
+      <c r="Z2" s="6" t="str">
         <v>Country</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="B3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="C3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="D3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="E3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="F3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="G3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="H3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="I3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="J3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="K3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="L3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="M3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="N3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="O3" s="5" t="str">
+      <c r="A3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="B3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="C3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="D3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="E3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="F3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="G3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="H3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="I3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="J3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="K3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="L3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="M3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="N3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="O3" s="6" t="str">
         <v>Num</v>
       </c>
-      <c r="P3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="Q3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="R3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="S3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="T3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="U3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="V3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="W3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="X3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="Y3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="Z3" s="5" t="str">
+      <c r="P3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="Q3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="R3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="S3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="T3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="U3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="V3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="W3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="X3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="Y3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="Z3" s="6" t="str">
         <v>Char</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="5">
+      <c r="A4" s="6">
         <v>12</v>
       </c>
-      <c r="B4" s="5">
+      <c r="B4" s="6">
         <v>2</v>
       </c>
-      <c r="C4" s="5">
+      <c r="C4" s="6">
         <v>8</v>
       </c>
-      <c r="D4" s="5">
+      <c r="D4" s="6">
         <v>4</v>
       </c>
-      <c r="E4" s="5">
+      <c r="E4" s="6">
         <v>10</v>
       </c>
-      <c r="F4" s="5">
+      <c r="F4" s="6">
         <v>10</v>
       </c>
-      <c r="G4" s="5">
+      <c r="G4" s="6">
         <v>10</v>
       </c>
-      <c r="H4" s="5">
+      <c r="H4" s="6">
         <v>10</v>
       </c>
-      <c r="I4" s="5">
+      <c r="I4" s="6">
         <v>10</v>
       </c>
-      <c r="J4" s="5">
+      <c r="J4" s="6">
         <v>10</v>
       </c>
-      <c r="K4" s="5">
+      <c r="K4" s="6">
         <v>10</v>
       </c>
-      <c r="L4" s="5">
+      <c r="L4" s="6">
         <v>1</v>
       </c>
-      <c r="M4" s="5">
+      <c r="M4" s="6">
         <v>3</v>
       </c>
-      <c r="N4" s="5">
+      <c r="N4" s="6">
         <v>10</v>
       </c>
-      <c r="O4" s="5">
+      <c r="O4" s="6">
         <v>8</v>
       </c>
-      <c r="P4" s="5">
+      <c r="P4" s="6">
         <v>5</v>
       </c>
-      <c r="Q4" s="5">
+      <c r="Q4" s="6">
         <v>1</v>
       </c>
-      <c r="R4" s="5">
+      <c r="R4" s="6">
         <v>41</v>
       </c>
-      <c r="S4" s="5">
+      <c r="S4" s="6">
         <v>22</v>
       </c>
-      <c r="T4" s="5">
+      <c r="T4" s="6">
         <v>8</v>
       </c>
-      <c r="U4" s="5">
+      <c r="U4" s="6">
         <v>28</v>
       </c>
-      <c r="V4" s="5">
+      <c r="V4" s="6">
         <v>8</v>
       </c>
-      <c r="W4" s="5">
+      <c r="W4" s="6">
         <v>28</v>
       </c>
-      <c r="X4" s="5">
+      <c r="X4" s="6">
         <v>14</v>
       </c>
-      <c r="Y4" s="5">
+      <c r="Y4" s="6">
         <v>200</v>
       </c>
-      <c r="Z4" s="5">
+      <c r="Z4" s="6">
         <v>3</v>
       </c>
     </row>
@@ -1023,7 +1046,7 @@
       <c r="D5" s="4">
         <v>1115</v>
       </c>
-      <c r="E5" s="6" t="str">
+      <c r="E5" s="7" t="str">
         <v/>
       </c>
       <c r="F5" s="4" t="str">
@@ -1183,7 +1206,7 @@
       <c r="D7" s="4">
         <v>1302</v>
       </c>
-      <c r="E7" s="6" t="str">
+      <c r="E7" s="8" t="str">
         <v/>
       </c>
       <c r="F7" s="4" t="str">
@@ -1343,7 +1366,7 @@
       <c r="D9" s="4">
         <v>1383</v>
       </c>
-      <c r="E9" s="6" t="str">
+      <c r="E9" s="8" t="str">
         <v/>
       </c>
       <c r="F9" s="4" t="str">
@@ -1663,7 +1686,7 @@
       <c r="D13" s="4">
         <v>1087</v>
       </c>
-      <c r="E13" s="6" t="str">
+      <c r="E13" s="8" t="str">
         <v/>
       </c>
       <c r="F13" s="4" t="str">
@@ -1875,161 +1898,161 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="5" t="str">
+      <c r="A2" s="6" t="str">
         <v>Study Identifier</v>
       </c>
-      <c r="B2" s="5" t="str">
+      <c r="B2" s="6" t="str">
         <v>Domain Abbreviation</v>
       </c>
-      <c r="C2" s="5" t="str">
+      <c r="C2" s="6" t="str">
         <v>Unique Subject Identifier</v>
       </c>
-      <c r="D2" s="5" t="str">
+      <c r="D2" s="6" t="str">
         <v>Sequence Number</v>
       </c>
-      <c r="E2" s="5" t="str">
+      <c r="E2" s="6" t="str">
         <v>Reported Name of Drug, Med, or Therapy</v>
       </c>
-      <c r="F2" s="5" t="str">
+      <c r="F2" s="6" t="str">
         <v>Indication</v>
       </c>
-      <c r="G2" s="5" t="str">
+      <c r="G2" s="6" t="str">
         <v>Dose per Administration</v>
       </c>
-      <c r="H2" s="5" t="str">
+      <c r="H2" s="6" t="str">
         <v>Dose Units</v>
       </c>
-      <c r="I2" s="5" t="str">
+      <c r="I2" s="6" t="str">
         <v>Dosing Frequency per Interval</v>
       </c>
-      <c r="J2" s="5" t="str">
+      <c r="J2" s="6" t="str">
         <v>Route of Administration</v>
       </c>
-      <c r="K2" s="5" t="str">
+      <c r="K2" s="6" t="str">
         <v>Epoch</v>
       </c>
-      <c r="L2" s="5" t="str">
+      <c r="L2" s="6" t="str">
         <v>Start Date/Time of Medication</v>
       </c>
-      <c r="M2" s="5" t="str">
+      <c r="M2" s="6" t="str">
         <v>End Date/Time of Medication</v>
       </c>
-      <c r="N2" s="5" t="str">
+      <c r="N2" s="6" t="str">
         <v>Study Day of Start of Medication</v>
       </c>
-      <c r="O2" s="5" t="str">
+      <c r="O2" s="6" t="str">
         <v>Study Day of End of Medication</v>
       </c>
-      <c r="P2" s="5" t="str">
+      <c r="P2" s="6" t="str">
         <v>Start Relative to Reference Period</v>
       </c>
-      <c r="Q2" s="5" t="str">
+      <c r="Q2" s="6" t="str">
         <v>End Relative to Reference Period</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="B3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="C3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="D3" s="5" t="str">
+      <c r="A3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="B3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="C3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="D3" s="6" t="str">
         <v>Num</v>
       </c>
-      <c r="E3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="F3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="G3" s="5" t="str">
+      <c r="E3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="F3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="G3" s="6" t="str">
         <v>Num</v>
       </c>
-      <c r="H3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="I3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="J3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="K3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="L3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="M3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="N3" s="5" t="str">
+      <c r="H3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="I3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="J3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="K3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="L3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="M3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="N3" s="6" t="str">
         <v>Num</v>
       </c>
-      <c r="O3" s="5" t="str">
+      <c r="O3" s="6" t="str">
         <v>Num</v>
       </c>
-      <c r="P3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="Q3" s="5" t="str">
+      <c r="P3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="Q3" s="6" t="str">
         <v>Char</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="5">
+      <c r="A4" s="6">
         <v>12</v>
       </c>
-      <c r="B4" s="5">
+      <c r="B4" s="6">
         <v>2</v>
       </c>
-      <c r="C4" s="5">
+      <c r="C4" s="6">
         <v>8</v>
       </c>
-      <c r="D4" s="5">
+      <c r="D4" s="6">
         <v>8</v>
       </c>
-      <c r="E4" s="5">
+      <c r="E4" s="6">
         <v>200</v>
       </c>
-      <c r="F4" s="5">
+      <c r="F4" s="6">
         <v>200</v>
       </c>
-      <c r="G4" s="5">
+      <c r="G4" s="6">
         <v>8</v>
       </c>
-      <c r="H4" s="5">
+      <c r="H4" s="6">
         <v>6</v>
       </c>
-      <c r="I4" s="5">
+      <c r="I4" s="6">
         <v>3</v>
       </c>
-      <c r="J4" s="5">
+      <c r="J4" s="6">
         <v>24</v>
       </c>
-      <c r="K4" s="5">
+      <c r="K4" s="6">
         <v>9</v>
       </c>
-      <c r="L4" s="5">
+      <c r="L4" s="6">
         <v>10</v>
       </c>
-      <c r="M4" s="5">
+      <c r="M4" s="6">
         <v>10</v>
       </c>
-      <c r="N4" s="5">
+      <c r="N4" s="6">
         <v>8</v>
       </c>
-      <c r="O4" s="5">
+      <c r="O4" s="6">
         <v>8</v>
       </c>
-      <c r="P4" s="5">
+      <c r="P4" s="6">
         <v>7</v>
       </c>
-      <c r="Q4" s="5">
+      <c r="Q4" s="6">
         <v>5</v>
       </c>
     </row>
@@ -2079,7 +2102,7 @@
       <c r="O5" s="4" t="str">
         <v/>
       </c>
-      <c r="P5" s="6" t="str">
+      <c r="P5" s="8" t="str">
         <v>ONGOING</v>
       </c>
       <c r="Q5" s="4" t="str">
@@ -2185,7 +2208,7 @@
       <c r="O7" s="4" t="str">
         <v/>
       </c>
-      <c r="P7" s="6" t="str">
+      <c r="P7" s="8" t="str">
         <v>ONGOING</v>
       </c>
       <c r="Q7" s="4" t="str">
@@ -2291,7 +2314,7 @@
       <c r="O9" s="4">
         <v>1</v>
       </c>
-      <c r="P9" s="6" t="str">
+      <c r="P9" s="8" t="str">
         <v>BEFORE</v>
       </c>
       <c r="Q9" s="4" t="str">
@@ -2503,7 +2526,7 @@
       <c r="O13" s="4">
         <v>181</v>
       </c>
-      <c r="P13" s="6" t="str">
+      <c r="P13" s="8" t="str">
         <v>AFTER</v>
       </c>
       <c r="Q13" s="4" t="str">

</xml_diff>